<commit_message>
Update HS summary: apply proportional trade discount to customs values
Discount factor 0.883055 (100229.39/113503.04) applied to all HS codes.
Adds pre/post-discount value columns. Total customs value = $100,229.39.

https://claude.ai/code/session_01SPn1SxbxU72qMQmioC8wGU
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Czech_Healthcare_196652.xlsx
+++ b/output/HS_Code_Summary_Czech_Healthcare_196652.xlsx
@@ -30,7 +30,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -41,6 +41,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
         <bgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+        <bgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -56,12 +62,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -427,18 +434,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="38" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -479,10 +487,15 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Celková hodnota (USD)</t>
+          <t>Celková hodnota (USD) – po slevě</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Celková hodnota (USD) – před slevou</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>TARIC ověření / poznámka</t>
         </is>
@@ -506,7 +519,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>FOB</t>
+          <t>FOB (nepotvrzeno)</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -516,6 +529,9 @@
         <v>792.3920000000001</v>
       </c>
       <c r="H2" t="n">
+        <v>29714.77</v>
+      </c>
+      <c r="I2" t="n">
         <v>33649.98</v>
       </c>
     </row>
@@ -537,7 +553,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>FOB</t>
+          <t>FOB (nepotvrzeno)</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -547,6 +563,9 @@
         <v>385.929</v>
       </c>
       <c r="H3" t="n">
+        <v>24561.75</v>
+      </c>
+      <c r="I3" t="n">
         <v>27814.53</v>
       </c>
     </row>
@@ -568,7 +587,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>FOB</t>
+          <t>FOB (nepotvrzeno)</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -578,6 +597,9 @@
         <v>741.196</v>
       </c>
       <c r="H4" t="n">
+        <v>8568.309999999999</v>
+      </c>
+      <c r="I4" t="n">
         <v>9703.040000000001</v>
       </c>
     </row>
@@ -599,7 +621,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>FOB</t>
+          <t>FOB (nepotvrzeno)</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -609,6 +631,9 @@
         <v>337.083</v>
       </c>
       <c r="H5" t="n">
+        <v>6376.8</v>
+      </c>
+      <c r="I5" t="n">
         <v>7221.3</v>
       </c>
     </row>
@@ -630,7 +655,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>FOB</t>
+          <t>FOB (nepotvrzeno)</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -640,6 +665,9 @@
         <v>387.365</v>
       </c>
       <c r="H6" t="n">
+        <v>5196.78</v>
+      </c>
+      <c r="I6" t="n">
         <v>5885</v>
       </c>
     </row>
@@ -661,7 +689,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>FOB</t>
+          <t>FOB (nepotvrzeno)</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -671,6 +699,9 @@
         <v>97.72799999999999</v>
       </c>
       <c r="H7" t="n">
+        <v>5033.45</v>
+      </c>
+      <c r="I7" t="n">
         <v>5700.04</v>
       </c>
     </row>
@@ -692,7 +723,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>FOB</t>
+          <t>FOB (nepotvrzeno)</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -702,6 +733,9 @@
         <v>59.592</v>
       </c>
       <c r="H8" t="n">
+        <v>3735.22</v>
+      </c>
+      <c r="I8" t="n">
         <v>4229.88</v>
       </c>
     </row>
@@ -723,7 +757,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>FOB</t>
+          <t>FOB (nepotvrzeno)</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -733,6 +767,9 @@
         <v>211.008</v>
       </c>
       <c r="H9" t="n">
+        <v>3448.58</v>
+      </c>
+      <c r="I9" t="n">
         <v>3905.28</v>
       </c>
     </row>
@@ -754,7 +791,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>FOB</t>
+          <t>FOB (nepotvrzeno)</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -764,6 +801,9 @@
         <v>41.976</v>
       </c>
       <c r="H10" t="n">
+        <v>2231.87</v>
+      </c>
+      <c r="I10" t="n">
         <v>2527.44</v>
       </c>
     </row>
@@ -785,7 +825,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>FOB</t>
+          <t>FOB (nepotvrzeno)</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -795,6 +835,9 @@
         <v>29.04</v>
       </c>
       <c r="H11" t="n">
+        <v>1990.05</v>
+      </c>
+      <c r="I11" t="n">
         <v>2253.6</v>
       </c>
     </row>
@@ -816,7 +859,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>FOB</t>
+          <t>FOB (nepotvrzeno)</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -826,6 +869,9 @@
         <v>90.536</v>
       </c>
       <c r="H12" t="n">
+        <v>1560.89</v>
+      </c>
+      <c r="I12" t="n">
         <v>1767.6</v>
       </c>
     </row>
@@ -847,7 +893,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>FOB</t>
+          <t>FOB (nepotvrzeno)</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -857,6 +903,9 @@
         <v>67.542</v>
       </c>
       <c r="H13" t="n">
+        <v>1110.74</v>
+      </c>
+      <c r="I13" t="n">
         <v>1257.84</v>
       </c>
     </row>
@@ -878,7 +927,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>FOB</t>
+          <t>FOB (nepotvrzeno)</t>
         </is>
       </c>
       <c r="E14" t="n">
@@ -888,6 +937,9 @@
         <v>21.232</v>
       </c>
       <c r="H14" t="n">
+        <v>867.9</v>
+      </c>
+      <c r="I14" t="n">
         <v>982.84</v>
       </c>
     </row>
@@ -909,7 +961,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>FOB</t>
+          <t>FOB (nepotvrzeno)</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -919,6 +971,9 @@
         <v>53.977</v>
       </c>
       <c r="H15" t="n">
+        <v>752.9299999999999</v>
+      </c>
+      <c r="I15" t="n">
         <v>852.64</v>
       </c>
     </row>
@@ -940,7 +995,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>FOB</t>
+          <t>FOB (nepotvrzeno)</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -950,6 +1005,9 @@
         <v>56.3</v>
       </c>
       <c r="H16" t="n">
+        <v>707.52</v>
+      </c>
+      <c r="I16" t="n">
         <v>801.22</v>
       </c>
     </row>
@@ -971,7 +1029,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>FOB</t>
+          <t>FOB (nepotvrzeno)</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -981,6 +1039,9 @@
         <v>3.216</v>
       </c>
       <c r="H17" t="n">
+        <v>551.45</v>
+      </c>
+      <c r="I17" t="n">
         <v>624.48</v>
       </c>
     </row>
@@ -1002,7 +1063,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>FOB</t>
+          <t>FOB (nepotvrzeno)</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -1012,6 +1073,9 @@
         <v>5.4</v>
       </c>
       <c r="H18" t="n">
+        <v>533.33</v>
+      </c>
+      <c r="I18" t="n">
         <v>603.96</v>
       </c>
     </row>
@@ -1033,7 +1097,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>FOB</t>
+          <t>FOB (nepotvrzeno)</t>
         </is>
       </c>
       <c r="E19" t="n">
@@ -1043,6 +1107,9 @@
         <v>15.54</v>
       </c>
       <c r="H19" t="n">
+        <v>505.04</v>
+      </c>
+      <c r="I19" t="n">
         <v>571.92</v>
       </c>
     </row>
@@ -1064,7 +1131,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>FOB</t>
+          <t>FOB (nepotvrzeno)</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -1074,6 +1141,9 @@
         <v>7.656</v>
       </c>
       <c r="H20" t="n">
+        <v>462.44</v>
+      </c>
+      <c r="I20" t="n">
         <v>523.6799999999999</v>
       </c>
     </row>
@@ -1095,7 +1165,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>FOB</t>
+          <t>FOB (nepotvrzeno)</t>
         </is>
       </c>
       <c r="E21" t="n">
@@ -1105,6 +1175,9 @@
         <v>12.924</v>
       </c>
       <c r="H21" t="n">
+        <v>424.24</v>
+      </c>
+      <c r="I21" t="n">
         <v>480.42</v>
       </c>
     </row>
@@ -1126,7 +1199,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>FOB</t>
+          <t>FOB (nepotvrzeno)</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -1136,6 +1209,9 @@
         <v>6.66</v>
       </c>
       <c r="H22" t="n">
+        <v>406.51</v>
+      </c>
+      <c r="I22" t="n">
         <v>460.35</v>
       </c>
     </row>
@@ -1157,7 +1233,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>FOB</t>
+          <t>FOB (nepotvrzeno)</t>
         </is>
       </c>
       <c r="E23" t="n">
@@ -1167,6 +1243,9 @@
         <v>8.1</v>
       </c>
       <c r="H23" t="n">
+        <v>382.35</v>
+      </c>
+      <c r="I23" t="n">
         <v>432.99</v>
       </c>
     </row>
@@ -1188,7 +1267,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>FOB</t>
+          <t>FOB (nepotvrzeno)</t>
         </is>
       </c>
       <c r="E24" t="n">
@@ -1198,6 +1277,9 @@
         <v>4.704</v>
       </c>
       <c r="H24" t="n">
+        <v>297.2</v>
+      </c>
+      <c r="I24" t="n">
         <v>336.56</v>
       </c>
     </row>
@@ -1219,7 +1301,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>FOB</t>
+          <t>FOB (nepotvrzeno)</t>
         </is>
       </c>
       <c r="E25" t="n">
@@ -1229,6 +1311,9 @@
         <v>3</v>
       </c>
       <c r="H25" t="n">
+        <v>203.99</v>
+      </c>
+      <c r="I25" t="n">
         <v>231</v>
       </c>
     </row>
@@ -1250,7 +1335,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>FOB</t>
+          <t>FOB (nepotvrzeno)</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -1260,6 +1345,9 @@
         <v>4.608</v>
       </c>
       <c r="H26" t="n">
+        <v>199.59</v>
+      </c>
+      <c r="I26" t="n">
         <v>226.02</v>
       </c>
     </row>
@@ -1281,7 +1369,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>FOB</t>
+          <t>FOB (nepotvrzeno)</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -1291,6 +1379,9 @@
         <v>6.237</v>
       </c>
       <c r="H27" t="n">
+        <v>176.87</v>
+      </c>
+      <c r="I27" t="n">
         <v>200.29</v>
       </c>
     </row>
@@ -1312,7 +1403,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>FOB</t>
+          <t>FOB (nepotvrzeno)</t>
         </is>
       </c>
       <c r="E28" t="n">
@@ -1322,6 +1413,9 @@
         <v>0.84</v>
       </c>
       <c r="H28" t="n">
+        <v>172.46</v>
+      </c>
+      <c r="I28" t="n">
         <v>195.3</v>
       </c>
     </row>
@@ -1343,7 +1437,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>FOB</t>
+          <t>FOB (nepotvrzeno)</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -1353,6 +1447,9 @@
         <v>3.864</v>
       </c>
       <c r="H29" t="n">
+        <v>56.37</v>
+      </c>
+      <c r="I29" t="n">
         <v>63.84</v>
       </c>
     </row>
@@ -1362,17 +1459,35 @@
           <t>CELKEM</t>
         </is>
       </c>
+      <c r="B30" s="2" t="n"/>
+      <c r="C30" s="2" t="n"/>
+      <c r="D30" s="2" t="n"/>
       <c r="E30" s="2" t="n">
         <v>5703</v>
       </c>
       <c r="F30" s="2" t="n">
         <v>3455.646</v>
       </c>
+      <c r="G30" s="2" t="n"/>
       <c r="H30" s="2" t="n">
+        <v>100229.39</v>
+      </c>
+      <c r="I30" s="2" t="n">
         <v>113503.04</v>
       </c>
+      <c r="J30" s="2" t="n"/>
+    </row>
+    <row r="31">
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>Sleva (Trade Discount z faktury): -$13,273.65 | Faktor: 0.883055</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="H31:I31"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1383,72 +1498,99 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="130" customWidth="1" min="1" max="1"/>
+    <col width="120" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Poznámky k souboru:</t>
+          <t>Poznámky k hodnotám:</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1) Incoterm: FOB – sloupec 'FOB' byl uveden v packing listu jako záhlaví (hodnota nebyla vyplněna), proto je FOB použit jako platný incoterm pro celou zásilku.</t>
+          <t>Faktura celkem (před slevou / hrubá hodnota): $113,503.04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2) Země původu (COO): zkontrolováno na úrovni jednotlivých položek (LINE ITEMS) – žádný HS kód nekombinuje více zemí původu. Všechny kódy mají jednu COO s výjimkou:</t>
+          <t>Faktura celkem (po slevě / čistá hodnota): $100,229.39</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - 3304995000 (kosmetika/lubrikant) -&gt; COO = US</t>
+          <t>Sleva: -$13,273.65 (Credit for RP Cords and Trade Discount – strana 7 faktury)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - 7325100080 (ocelové spekulum) -&gt; COO = PK</t>
+          <t>Koeficient přepočtu: 0.883055</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Všechny ostatní kódy -&gt; COO = CN.</t>
-        </is>
-      </c>
+      <c r="A6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>3) Celková hrubá hmotnost (kg): ponecháno prázdné na úrovni HS kódu, protože zdrojové dokumenty (BOL) uvádějí hrubou hmotnost pouze souhrnně za celou zásilku (3870,050 kg), nikoli po HS kódech. Bude doplněno později.</t>
+          <t>Sleva je paušální obchodní sleva na celou zásilku (strana 7 faktury SO-196652).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>4) Sloupec 'TARIC ověření / poznámka' je určen k označení HS kódů, které bude potřeba ručně ověřit/dohledat v databázi TARIC.</t>
+          <t>Celková výše slevy přesahuje hodnotu položek na straně 7, proto je rozpočítána proporcionálně na všechny HS kódy.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>5) Zdroj dat: HSCodeTotals__Czech_Healthcare_196652.xlsx (sheet TOTALS), zkříženo s Final_BOLSEJ2226.pdf (čistá hmotnost odpovídá 3455,646 kg) a Czech_Healthcare__PLwC_196652.pdf (FOB sloupec).</t>
+          <t>Sloupec 'Celková hodnota – po slevě' = hodnota pro celní deklaraci (transakční hodnota dle WTO).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Sloupec 'Celková hodnota – před slevou' = součet řádkových hodnot z faktury před slevou (pro referenci).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Incoterm: FOB – záhlaví sloupce v packing listu, hodnota buňky nevyplněna. Nutno potvrdit s dopravcem/dodavatelem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Hrubá hmotnost (kg) na úrovni HS kódu: nevyplněna – BOL uvádí pouze celkovou hrubou hmotnost zásilky (3870,050 kg).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>COO: zkontrolováno na úrovni položek – 3304995000 = US, 7325100080 = PK, ostatní = CN.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update HS code summary: gross weights, CBAM flags, antidumping note
- Fill gross weight column for all 28 HS codes (proportional: NW × 1.11992)
- Flag CBAM goods orange: 7326908688 (steel) and 7616995190 (aluminium), Y137 de minimis
- Flag antidumping red: 3406000000 (candles CN), duty amounts in notes
- Add pre/post-discount value columns (factor 0.883055)
- Add Dokumenty a poznámky sheet with document status and open issues

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SPn1SxbxU72qMQmioC8wGU
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Czech_Healthcare_196652.xlsx
+++ b/output/HS_Code_Summary_Czech_Healthcare_196652.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="HS Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Poznámky" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Dokumenty a poznámky" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,9 +28,30 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <sz val="9"/>
+    </font>
+    <font>
+      <color rgb="00006100"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="009C0006"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -39,14 +60,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
-        <bgColor rgb="00D9E1F2"/>
+        <fgColor rgb="001F4E79"/>
+        <bgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-        <bgColor rgb="00FFEB9C"/>
+        <fgColor rgb="00EBF3FB"/>
+        <bgColor rgb="00EBF3FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC000"/>
+        <bgColor rgb="00FFC000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF0000"/>
+        <bgColor rgb="00FF0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+        <bgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -62,13 +101,29 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -434,22 +489,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="55" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>HS kód</t>
@@ -477,1016 +533,1252 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Celková čistá hmotnost (kg)</t>
+          <t>Čistá hmotnost (kg)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Celková hrubá hmotnost (kg)</t>
+          <t>Hrubá hmotnost (kg)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Celková hodnota (USD) – po slevě</t>
+          <t>Hodnota USD – po slevě</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Celková hodnota (USD) – před slevou</t>
+          <t>Hodnota USD – před slevou</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>TARIC ověření / poznámka</t>
+          <t>Příznak</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>TARIC / poznámka / CBAM / Antidumping</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>3926909989</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Ostatní výrobky z plastů (erotické pomůcky)</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>FOB (nepotvrzeno)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
         <v>2411</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="2" t="n">
         <v>792.3920000000001</v>
       </c>
-      <c r="H2" t="n">
+      <c r="G2" s="2" t="n">
+        <v>887.415</v>
+      </c>
+      <c r="H2" s="2" t="n">
         <v>29714.77</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I2" s="2" t="n">
         <v>33649.98</v>
       </c>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>9019102010</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Masážní přístroje (vibrátory)</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>FOB (nepotvrzeno)</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="n">
         <v>1174</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="3" t="n">
         <v>385.929</v>
       </c>
-      <c r="H3" t="n">
+      <c r="G3" s="3" t="n">
+        <v>432.209</v>
+      </c>
+      <c r="H3" s="3" t="n">
         <v>24561.75</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I3" s="3" t="n">
         <v>27814.53</v>
       </c>
+      <c r="J3" s="3" t="inlineStr"/>
+      <c r="K3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>9019102035</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Masážní přístroje – sety s nábytkem</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>FOB (nepotvrzeno)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="2" t="n">
         <v>741.196</v>
       </c>
-      <c r="H4" t="n">
+      <c r="G4" s="2" t="n">
+        <v>830.08</v>
+      </c>
+      <c r="H4" s="2" t="n">
         <v>8568.309999999999</v>
       </c>
-      <c r="I4" t="n">
+      <c r="I4" s="2" t="n">
         <v>9703.040000000001</v>
       </c>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>6307909891</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Textilní doplňky (postroje)</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>FOB (nepotvrzeno)</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="n">
         <v>283</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="3" t="n">
         <v>337.083</v>
       </c>
-      <c r="H5" t="n">
+      <c r="G5" s="3" t="n">
+        <v>377.506</v>
+      </c>
+      <c r="H5" s="3" t="n">
         <v>6376.8</v>
       </c>
-      <c r="I5" t="n">
+      <c r="I5" s="3" t="n">
         <v>7221.3</v>
       </c>
+      <c r="J5" s="3" t="inlineStr"/>
+      <c r="K5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>9401710011</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Čalouněný sedací nábytek (kovová kostra)</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>FOB (nepotvrzeno)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="2" t="n">
         <v>387.365</v>
       </c>
-      <c r="H6" t="n">
+      <c r="G6" s="2" t="n">
+        <v>433.818</v>
+      </c>
+      <c r="H6" s="2" t="n">
         <v>5196.78</v>
       </c>
-      <c r="I6" t="n">
+      <c r="I6" s="2" t="n">
         <v>5885</v>
       </c>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>3926902100</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Plastové hygienické potřeby (klystýry)</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>FOB (nepotvrzeno)</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="n">
         <v>512</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="3" t="n">
         <v>97.72799999999999</v>
       </c>
-      <c r="H7" t="n">
+      <c r="G7" s="3" t="n">
+        <v>109.447</v>
+      </c>
+      <c r="H7" s="3" t="n">
         <v>5033.45</v>
       </c>
-      <c r="I7" t="n">
+      <c r="I7" s="3" t="n">
         <v>5700.04</v>
       </c>
+      <c r="J7" s="3" t="inlineStr"/>
+      <c r="K7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>7326908688</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Kovové výrobky z oceli (anální nástroje)</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>FOB (nepotvrzeno)</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="n">
         <v>180</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8" s="4" t="n">
         <v>59.592</v>
       </c>
-      <c r="H8" t="n">
+      <c r="G8" s="4" t="n">
+        <v>66.738</v>
+      </c>
+      <c r="H8" s="4" t="n">
         <v>3735.22</v>
       </c>
-      <c r="I8" t="n">
+      <c r="I8" s="4" t="n">
         <v>4229.88</v>
       </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>CBAM</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>CBAM zboží (železo/ocel). Zákazník uplatňuje výjimku de minimis (kód Y137) – dovoz v řádu desítek kg, pod limitem 50 t/rok.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>6301900030</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Přikrývky (deky)</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>FOB (nepotvrzeno)</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="n">
         <v>96</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9" s="3" t="n">
         <v>211.008</v>
       </c>
-      <c r="H9" t="n">
+      <c r="G9" s="3" t="n">
+        <v>236.312</v>
+      </c>
+      <c r="H9" s="3" t="n">
         <v>3448.58</v>
       </c>
-      <c r="I9" t="n">
+      <c r="I9" s="3" t="n">
         <v>3905.28</v>
       </c>
+      <c r="J9" s="3" t="inlineStr"/>
+      <c r="K9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>8414100000</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Vývěvy (penis pumpy)</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>FOB (nepotvrzeno)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10" s="2" t="n">
         <v>41.976</v>
       </c>
-      <c r="H10" t="n">
+      <c r="G10" s="2" t="n">
+        <v>47.01</v>
+      </c>
+      <c r="H10" s="2" t="n">
         <v>2231.87</v>
       </c>
-      <c r="I10" t="n">
+      <c r="I10" s="2" t="n">
         <v>2527.44</v>
       </c>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>7907006000</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Výrobky ze zinku (popruhy)</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>FOB (nepotvrzeno)</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="n">
         <v>240</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F11" s="3" t="n">
         <v>29.04</v>
       </c>
-      <c r="H11" t="n">
+      <c r="G11" s="3" t="n">
+        <v>32.522</v>
+      </c>
+      <c r="H11" s="3" t="n">
         <v>1990.05</v>
       </c>
-      <c r="I11" t="n">
+      <c r="I11" s="3" t="n">
         <v>2253.6</v>
       </c>
+      <c r="J11" s="3" t="inlineStr"/>
+      <c r="K11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>3304995000</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Kosmetické přípravky (lubrikant)</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>FOB (nepotvrzeno)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F12" s="2" t="n">
         <v>90.536</v>
       </c>
-      <c r="H12" t="n">
+      <c r="G12" s="2" t="n">
+        <v>101.393</v>
+      </c>
+      <c r="H12" s="2" t="n">
         <v>1560.89</v>
       </c>
-      <c r="I12" t="n">
+      <c r="I12" s="2" t="n">
         <v>1767.6</v>
       </c>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>9506996080</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Sportovní potřeby (sex stoličky)</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>FOB (nepotvrzeno)</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F13" s="3" t="n">
         <v>67.542</v>
       </c>
-      <c r="H13" t="n">
+      <c r="G13" s="3" t="n">
+        <v>75.642</v>
+      </c>
+      <c r="H13" s="3" t="n">
         <v>1110.74</v>
       </c>
-      <c r="I13" t="n">
+      <c r="I13" s="3" t="n">
         <v>1257.84</v>
       </c>
+      <c r="J13" s="3" t="inlineStr"/>
+      <c r="K13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>7020006000</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>Skleněné výrobky (dilda)</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>FOB (nepotvrzeno)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="n">
         <v>92</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F14" s="2" t="n">
         <v>21.232</v>
       </c>
-      <c r="H14" t="n">
+      <c r="G14" s="2" t="n">
+        <v>23.778</v>
+      </c>
+      <c r="H14" s="2" t="n">
         <v>867.9</v>
       </c>
-      <c r="I14" t="n">
+      <c r="I14" s="2" t="n">
         <v>982.84</v>
       </c>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>9403509080</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Dřevěný nábytek (bondage stůl)</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>FOB (nepotvrzeno)</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F15" t="n">
+      <c r="F15" s="3" t="n">
         <v>53.977</v>
       </c>
-      <c r="H15" t="n">
+      <c r="G15" s="3" t="n">
+        <v>60.45</v>
+      </c>
+      <c r="H15" s="3" t="n">
         <v>752.9299999999999</v>
       </c>
-      <c r="I15" t="n">
+      <c r="I15" s="3" t="n">
         <v>852.64</v>
       </c>
+      <c r="J15" s="3" t="inlineStr"/>
+      <c r="K15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>9401616011</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>Čalouněná sedadla s dřevěnou kostrou</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>FOB (nepotvrzeno)</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="F16" t="n">
+      <c r="F16" s="2" t="n">
         <v>56.3</v>
       </c>
-      <c r="H16" t="n">
+      <c r="G16" s="2" t="n">
+        <v>63.051</v>
+      </c>
+      <c r="H16" s="2" t="n">
         <v>707.52</v>
       </c>
-      <c r="I16" t="n">
+      <c r="I16" s="2" t="n">
         <v>801.22</v>
       </c>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>6505009089</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>Pokrývky hlavy (masky)</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E17" t="n">
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>FOB (nepotvrzeno)</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="n">
         <v>72</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F17" s="3" t="n">
         <v>3.216</v>
       </c>
-      <c r="H17" t="n">
+      <c r="G17" s="3" t="n">
+        <v>3.602</v>
+      </c>
+      <c r="H17" s="3" t="n">
         <v>551.45</v>
       </c>
-      <c r="I17" t="n">
+      <c r="I17" s="3" t="n">
         <v>624.48</v>
       </c>
+      <c r="J17" s="3" t="inlineStr"/>
+      <c r="K17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>8205700060</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>Ruční nástroje (klipy na bradavky)</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E18" t="n">
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>FOB (nepotvrzeno)</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n">
         <v>84</v>
       </c>
-      <c r="F18" t="n">
+      <c r="F18" s="2" t="n">
         <v>5.4</v>
       </c>
-      <c r="H18" t="n">
+      <c r="G18" s="2" t="n">
+        <v>6.048</v>
+      </c>
+      <c r="H18" s="2" t="n">
         <v>533.33</v>
       </c>
-      <c r="I18" t="n">
+      <c r="I18" s="2" t="n">
         <v>603.96</v>
       </c>
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>3406000000</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>Svíčky</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>FOB (nepotvrzeno)</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="n">
         <v>120</v>
       </c>
-      <c r="F19" t="n">
+      <c r="F19" s="5" t="n">
         <v>15.54</v>
       </c>
-      <c r="H19" t="n">
+      <c r="G19" s="5" t="n">
+        <v>17.404</v>
+      </c>
+      <c r="H19" s="5" t="n">
         <v>505.04</v>
       </c>
-      <c r="I19" t="n">
+      <c r="I19" s="5" t="n">
         <v>571.92</v>
       </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>ANTIDUMPING</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>Antidumpingové clo z CN! Základ A00: 11 990 CZK @ 60,3% = 7 230 CZK + základ 19 220 CZK @ 21% = 2 518 CZK. Ověřit výši při podání JSD.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>6602000000</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>Biče a švihadla</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E20" t="n">
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>FOB (nepotvrzeno)</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="F20" t="n">
+      <c r="F20" s="2" t="n">
         <v>7.656</v>
       </c>
-      <c r="H20" t="n">
+      <c r="G20" s="2" t="n">
+        <v>8.574</v>
+      </c>
+      <c r="H20" s="2" t="n">
         <v>462.44</v>
       </c>
-      <c r="I20" t="n">
+      <c r="I20" s="2" t="n">
         <v>523.6799999999999</v>
       </c>
+      <c r="J20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>9020006000</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Dýchací přístroje (masky)</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E21" t="n">
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>FOB (nepotvrzeno)</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="F21" t="n">
+      <c r="F21" s="3" t="n">
         <v>12.924</v>
       </c>
-      <c r="H21" t="n">
+      <c r="G21" s="3" t="n">
+        <v>14.474</v>
+      </c>
+      <c r="H21" s="3" t="n">
         <v>424.24</v>
       </c>
-      <c r="I21" t="n">
+      <c r="I21" s="3" t="n">
         <v>480.42</v>
       </c>
+      <c r="J21" s="3" t="inlineStr"/>
+      <c r="K21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>7325100080</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>Odlitky z oceli (spekulum)</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E22" t="n">
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>FOB (nepotvrzeno)</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="F22" t="n">
+      <c r="F22" s="2" t="n">
         <v>6.66</v>
       </c>
-      <c r="H22" t="n">
+      <c r="G22" s="2" t="n">
+        <v>7.459</v>
+      </c>
+      <c r="H22" s="2" t="n">
         <v>406.51</v>
       </c>
-      <c r="I22" t="n">
+      <c r="I22" s="2" t="n">
         <v>460.35</v>
       </c>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>9404902090</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>Lůžkoviny (polštáře)</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E23" t="n">
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>FOB (nepotvrzeno)</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="F23" t="n">
+      <c r="F23" s="3" t="n">
         <v>8.1</v>
       </c>
-      <c r="H23" t="n">
+      <c r="G23" s="3" t="n">
+        <v>9.071</v>
+      </c>
+      <c r="H23" s="3" t="n">
         <v>382.35</v>
       </c>
-      <c r="I23" t="n">
+      <c r="I23" s="3" t="n">
         <v>432.99</v>
       </c>
+      <c r="J23" s="3" t="inlineStr"/>
+      <c r="K23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>7616995190</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>Výrobky z hliníku (kolíky)</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E24" t="n">
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>FOB (nepotvrzeno)</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="n">
         <v>56</v>
       </c>
-      <c r="F24" t="n">
+      <c r="F24" s="4" t="n">
         <v>4.704</v>
       </c>
-      <c r="H24" t="n">
+      <c r="G24" s="4" t="n">
+        <v>5.268</v>
+      </c>
+      <c r="H24" s="4" t="n">
         <v>297.2</v>
       </c>
-      <c r="I24" t="n">
+      <c r="I24" s="4" t="n">
         <v>336.56</v>
       </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>CBAM</t>
+        </is>
+      </c>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>CBAM zboží (hliník). Zákazník uplatňuje výjimku de minimis (kód Y137) – dovoz v řádu desítek kg, pod limitem 50 t/rok.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>8543709860</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>Elektrické přístroje (e-stim)</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E25" t="n">
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>FOB (nepotvrzeno)</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="F25" t="n">
+      <c r="F25" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="H25" t="n">
+      <c r="G25" s="3" t="n">
+        <v>3.36</v>
+      </c>
+      <c r="H25" s="3" t="n">
         <v>203.99</v>
       </c>
-      <c r="I25" t="n">
+      <c r="I25" s="3" t="n">
         <v>231</v>
       </c>
+      <c r="J25" s="3" t="inlineStr"/>
+      <c r="K25" s="3" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>9503000090</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>Hračky (plyšáci, pouta)</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E26" t="n">
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>FOB (nepotvrzeno)</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="F26" t="n">
+      <c r="F26" s="2" t="n">
         <v>4.608</v>
       </c>
-      <c r="H26" t="n">
+      <c r="G26" s="2" t="n">
+        <v>5.161</v>
+      </c>
+      <c r="H26" s="2" t="n">
         <v>199.59</v>
       </c>
-      <c r="I26" t="n">
+      <c r="I26" s="2" t="n">
         <v>226.02</v>
       </c>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>9401790050</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>Ostatní sedadla</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E27" t="n">
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>FOB (nepotvrzeno)</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="F27" t="n">
+      <c r="F27" s="3" t="n">
         <v>6.237</v>
       </c>
-      <c r="H27" t="n">
+      <c r="G27" s="3" t="n">
+        <v>6.985</v>
+      </c>
+      <c r="H27" s="3" t="n">
         <v>176.87</v>
       </c>
-      <c r="I27" t="n">
+      <c r="I27" s="3" t="n">
         <v>200.29</v>
       </c>
+      <c r="J27" s="3" t="inlineStr"/>
+      <c r="K27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>8505110090</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>Magnety (magnetické kuličky)</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E28" t="n">
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>FOB (nepotvrzeno)</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="F28" t="n">
+      <c r="F28" s="2" t="n">
         <v>0.84</v>
       </c>
-      <c r="H28" t="n">
+      <c r="G28" s="2" t="n">
+        <v>0.9409999999999999</v>
+      </c>
+      <c r="H28" s="2" t="n">
         <v>172.46</v>
       </c>
-      <c r="I28" t="n">
+      <c r="I28" s="2" t="n">
         <v>195.3</v>
       </c>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>3401115000</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>Mýdlo</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E29" t="n">
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>FOB (nepotvrzeno)</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="F29" t="n">
+      <c r="F29" s="3" t="n">
         <v>3.864</v>
       </c>
-      <c r="H29" t="n">
+      <c r="G29" s="3" t="n">
+        <v>4.327</v>
+      </c>
+      <c r="H29" s="3" t="n">
         <v>56.37</v>
       </c>
-      <c r="I29" t="n">
+      <c r="I29" s="3" t="n">
         <v>63.84</v>
       </c>
+      <c r="J29" s="3" t="inlineStr"/>
+      <c r="K29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="A30" s="6" t="inlineStr">
         <is>
           <t>CELKEM</t>
         </is>
       </c>
-      <c r="B30" s="2" t="n"/>
-      <c r="C30" s="2" t="n"/>
-      <c r="D30" s="2" t="n"/>
-      <c r="E30" s="2" t="n">
+      <c r="B30" s="6" t="n"/>
+      <c r="C30" s="6" t="n"/>
+      <c r="D30" s="6" t="n"/>
+      <c r="E30" s="6" t="n">
         <v>5703</v>
       </c>
-      <c r="F30" s="2" t="n">
+      <c r="F30" s="6" t="n">
         <v>3455.646</v>
       </c>
-      <c r="G30" s="2" t="n"/>
-      <c r="H30" s="2" t="n">
+      <c r="G30" s="6" t="n">
+        <v>3870.045</v>
+      </c>
+      <c r="H30" s="6" t="n">
         <v>100229.39</v>
       </c>
-      <c r="I30" s="2" t="n">
+      <c r="I30" s="6" t="n">
         <v>113503.04</v>
       </c>
-      <c r="J30" s="2" t="n"/>
-    </row>
-    <row r="31">
-      <c r="H31" s="3" t="inlineStr">
-        <is>
-          <t>Sleva (Trade Discount z faktury): -$13,273.65 | Faktor: 0.883055</t>
+      <c r="J30" s="6" t="n"/>
+      <c r="K30" s="6" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>Legenda:</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>🟡 ORANŽOVÁ</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>CBAM zboží – nutno uvést kód Y137 (de minimis výjimka) v JSD</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>🔴 ČERVENÁ</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>Antidumpingové clo – nutno zkontrolovat a uvést v JSD</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>FOB (nepotvrzeno)</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>Incoterm nebyl výslovně uveden v dokumentech – potvrdit s dodavatelem</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>Hrubá hmotnost</t>
+        </is>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>Vypočtena proporcionálně: čistá hmotnost × 1.11992 (celková GW 3870.05 / celková NW 3455.65)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>Sleva</t>
+        </is>
+      </c>
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>Obchodní sleva –$13 273,65 z faktury str. 7, faktor 0.883055</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="H31:I31"/>
+  <mergeCells count="5">
+    <mergeCell ref="B35:K35"/>
+    <mergeCell ref="B34:K34"/>
+    <mergeCell ref="B33:K33"/>
+    <mergeCell ref="B36:K36"/>
+    <mergeCell ref="B37:K37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1498,99 +1790,170 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="120" customWidth="1" min="1" max="1"/>
+    <col width="130" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Poznámky k hodnotám:</t>
-        </is>
+      <c r="A1" s="7">
+        <f>== PŘIJATÉ DOKUMENTY (stav 22.6.2026) ===</f>
+        <v/>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Faktura celkem (před slevou / hrubá hodnota): $113,503.04</t>
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>✓ Plná moc k přímému zastoupení – Czech Healthcare s.r.o. → Maurice Ward &amp; Co., podepsána 21.6.2026</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Faktura celkem (po slevě / čistá hodnota): $100,229.39</t>
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>✓ Plná moc k nepřímému zastoupení – Czech Healthcare s.r.o. → Maurice Ward &amp; Co., podepsána 21.6.2026</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Sleva: -$13,273.65 (Credit for RP Cords and Trade Discount – strana 7 faktury)</t>
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>✓ Čestné prohlášení o obalech – Czech Healthcare deklaruje splnění §15a zák. o obalech (méně než 300 kg/rok, obrat pod 25 mil. Kč), nepodléhá registraci zpětného odběru. Podepsáno 21.6.2026.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Koeficient přepočtu: 0.883055</t>
-        </is>
-      </c>
+      <c r="A5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
+      <c r="A6" s="7">
+        <f>== CBAM ===</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Sleva je paušální obchodní sleva na celou zásilku (strana 7 faktury SO-196652).</t>
+          <t>Dotčené HS kódy: 7326908688 (železo/ocel, 59,592 kg NW) a 7616995190 (hliník, 4,704 kg NW).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Celková výše slevy přesahuje hodnotu položek na straně 7, proto je rozpočítána proporcionálně na všechny HS kódy.</t>
+          <t>Celková čistá hmotnost CBAM zboží v zásilce: cca 64,3 kg – VÝRAZNĚ pod limitem 50 t/rok.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Sloupec 'Celková hodnota – po slevě' = hodnota pro celní deklaraci (transakční hodnota dle WTO).</t>
+          <t>Zákazník potvrdil: 'Uplatňujeme výjimku de minimis. Naše importy se pohybují v desítkách kg.'</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Sloupec 'Celková hodnota – před slevou' = součet řádkových hodnot z faktury před slevou (pro referenci).</t>
+          <t>→ Do JSD uvést kód Y137 (výjimka de minimis CBAM) u obou dotčených HS kódů.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Alternativy Y238 (žádost o schváleného deklaranta) a Y128 (přidělený status) NEPLATÍ – zákazník neuváděl.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Incoterm: FOB – záhlaví sloupce v packing listu, hodnota buňky nevyplněna. Nutno potvrdit s dopravcem/dodavatelem.</t>
-        </is>
-      </c>
+      <c r="A12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Hrubá hmotnost (kg) na úrovni HS kódu: nevyplněna – BOL uvádí pouze celkovou hrubou hmotnost zásilky (3870,050 kg).</t>
-        </is>
+      <c r="A13" s="7">
+        <f>== ANTIDUMPING – 3406000000 (svíčky, CN) ===</f>
+        <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>COO: zkontrolováno na úrovni položek – 3304995000 = US, 7325100080 = PK, ostatní = CN.</t>
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>Platí antidumpingové clo na svíčky z ČLR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Základ A00: 11 990 CZK @ sazba 60,3 % = 7 230 CZK</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Základ: 19 220 CZK @ sazba 21 % = 2 518 CZK</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Hodnota svíček v zásilce: $504,96 (po slevě). Ověřit základ cla při podání JSD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="7">
+        <f>== INCOTERM ===</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Sloupec FOB existuje v packing listu jako záhlaví, ale hodnota není vyplněna.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Prodejce ani dopravce incoterm výslovně nepotvrdil. → Potvrdit s XR Brands / Maurice Ward před podáním.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="7">
+        <f>== HMOTNOSTI ===</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Čistá hmotnost celkem: 3455.65 kg (ověřeno z nového PL i BOL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Hrubá hmotnost celkem: 3870.05 kg (BOL + nový PL, str. 31: packaging 15× 27,63 kg = 414,4 kg)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Hrubá hmotnost na úrovni HS kódu: proporcionální výpočet, faktor 1.11992</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix: merge 9019 rows to 27 HS codes, remove Incoterm column
- Merge 9019102010 + 9019102035 → single row 9019109000 (matches Helios)
- Remove Incoterm column per user request

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SPn1SxbxU72qMQmioC8wGU
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Czech_Healthcare_196652.xlsx
+++ b/output/HS_Code_Summary_Czech_Healthcare_196652.xlsx
@@ -489,20 +489,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K37"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="55" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="55" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -523,40 +522,35 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Incoterm</t>
+          <t>Celkové množství (ks)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Celkové množství (ks)</t>
+          <t>Čistá hmotnost (kg)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Čistá hmotnost (kg)</t>
+          <t>Hrubá hmotnost (kg)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Hrubá hmotnost (kg)</t>
+          <t>Hodnota USD – po slevě</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Hodnota USD – po slevě</t>
+          <t>Hodnota USD – před slevou</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Hodnota USD – před slevou</t>
+          <t>Příznak</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Příznak</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>TARIC / poznámka / CBAM / Antidumping</t>
         </is>
@@ -578,33 +572,28 @@
           <t>CN</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
+      <c r="D2" s="2" t="n">
+        <v>2411</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>2411</v>
+        <v>792.3920000000001</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>792.3920000000001</v>
+        <v>887.415</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>887.415</v>
+        <v>29714.77</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>29714.77</v>
-      </c>
-      <c r="I2" s="2" t="n">
         <v>33649.98</v>
       </c>
+      <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>9019102010</t>
+          <t>9019109000</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -617,38 +606,33 @@
           <t>CN</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
+      <c r="D3" s="3" t="n">
+        <v>1190</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>1174</v>
+        <v>1127.125</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>385.929</v>
+        <v>1262.289</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>432.209</v>
+        <v>33130.07</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>24561.75</v>
-      </c>
-      <c r="I3" s="3" t="n">
-        <v>27814.53</v>
-      </c>
+        <v>37517.57</v>
+      </c>
+      <c r="I3" s="3" t="inlineStr"/>
       <c r="J3" s="3" t="inlineStr"/>
-      <c r="K3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>9019102035</t>
+          <t>6307909891</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Masážní přístroje – sety s nábytkem</t>
+          <t>Textilní doplňky (postroje)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -656,38 +640,33 @@
           <t>CN</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
+      <c r="D4" s="2" t="n">
+        <v>283</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>16</v>
+        <v>337.083</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>741.196</v>
+        <v>377.506</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>830.08</v>
+        <v>6376.8</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>8568.309999999999</v>
-      </c>
-      <c r="I4" s="2" t="n">
-        <v>9703.040000000001</v>
-      </c>
+        <v>7221.3</v>
+      </c>
+      <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>6307909891</t>
+          <t>9401710011</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Textilní doplňky (postroje)</t>
+          <t>Čalouněný sedací nábytek (kovová kostra)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -695,38 +674,33 @@
           <t>CN</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
+      <c r="D5" s="3" t="n">
+        <v>14</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>283</v>
+        <v>387.365</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>337.083</v>
+        <v>433.818</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>377.506</v>
+        <v>5196.78</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>6376.8</v>
-      </c>
-      <c r="I5" s="3" t="n">
-        <v>7221.3</v>
-      </c>
+        <v>5885</v>
+      </c>
+      <c r="I5" s="3" t="inlineStr"/>
       <c r="J5" s="3" t="inlineStr"/>
-      <c r="K5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>9401710011</t>
+          <t>3926902100</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Čalouněný sedací nábytek (kovová kostra)</t>
+          <t>Plastové hygienické potřeby (klystýry)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -734,124 +708,109 @@
           <t>CN</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
+      <c r="D6" s="2" t="n">
+        <v>512</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>14</v>
+        <v>97.72799999999999</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>387.365</v>
+        <v>109.447</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>433.818</v>
+        <v>5033.45</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>5196.78</v>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>5885</v>
-      </c>
+        <v>5700.04</v>
+      </c>
+      <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>3926902100</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Plastové hygienické potřeby (klystýry)</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>512</v>
-      </c>
-      <c r="F7" s="3" t="n">
-        <v>97.72799999999999</v>
-      </c>
-      <c r="G7" s="3" t="n">
-        <v>109.447</v>
-      </c>
-      <c r="H7" s="3" t="n">
-        <v>5033.45</v>
-      </c>
-      <c r="I7" s="3" t="n">
-        <v>5700.04</v>
-      </c>
-      <c r="J7" s="3" t="inlineStr"/>
-      <c r="K7" s="3" t="inlineStr"/>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>7326908688</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Kovové výrobky z oceli (anální nástroje)</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>180</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>59.592</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>66.738</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>3735.22</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>4229.88</v>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>CBAM</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>CBAM zboží (železo/ocel). Zákazník uplatňuje výjimku de minimis (kód Y137) – dovoz v řádu desítek kg, pod limitem 50 t/rok.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>7326908688</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Kovové výrobky z oceli (anální nástroje)</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="n">
-        <v>180</v>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>59.592</v>
-      </c>
-      <c r="G8" s="4" t="n">
-        <v>66.738</v>
-      </c>
-      <c r="H8" s="4" t="n">
-        <v>3735.22</v>
-      </c>
-      <c r="I8" s="4" t="n">
-        <v>4229.88</v>
-      </c>
-      <c r="J8" s="4" t="inlineStr">
-        <is>
-          <t>CBAM</t>
-        </is>
-      </c>
-      <c r="K8" s="4" t="inlineStr">
-        <is>
-          <t>CBAM zboží (železo/ocel). Zákazník uplatňuje výjimku de minimis (kód Y137) – dovoz v řádu desítek kg, pod limitem 50 t/rok.</t>
-        </is>
-      </c>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>6301900030</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Přikrývky (deky)</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>211.008</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>236.312</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>3448.58</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>3905.28</v>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>6301900030</t>
+          <t>8414100000</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Přikrývky (deky)</t>
+          <t>Vývěvy (penis pumpy)</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -859,38 +818,33 @@
           <t>CN</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
+      <c r="D9" s="3" t="n">
+        <v>60</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>96</v>
+        <v>41.976</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>211.008</v>
+        <v>47.01</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>236.312</v>
+        <v>2231.87</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>3448.58</v>
-      </c>
-      <c r="I9" s="3" t="n">
-        <v>3905.28</v>
-      </c>
+        <v>2527.44</v>
+      </c>
+      <c r="I9" s="3" t="inlineStr"/>
       <c r="J9" s="3" t="inlineStr"/>
-      <c r="K9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>8414100000</t>
+          <t>7907006000</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Vývěvy (penis pumpy)</t>
+          <t>Výrobky ze zinku (popruhy)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -898,116 +852,101 @@
           <t>CN</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
+      <c r="D10" s="2" t="n">
+        <v>240</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>60</v>
+        <v>29.04</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>41.976</v>
+        <v>32.522</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>47.01</v>
+        <v>1990.05</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>2231.87</v>
-      </c>
-      <c r="I10" s="2" t="n">
-        <v>2527.44</v>
-      </c>
+        <v>2253.6</v>
+      </c>
+      <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr"/>
-      <c r="K10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>7907006000</t>
+          <t>3304995000</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Výrobky ze zinku (popruhy)</t>
+          <t>Kosmetické přípravky (lubrikant)</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>120</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>240</v>
+        <v>90.536</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>29.04</v>
+        <v>101.393</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>32.522</v>
+        <v>1560.89</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>1990.05</v>
-      </c>
-      <c r="I11" s="3" t="n">
-        <v>2253.6</v>
-      </c>
+        <v>1767.6</v>
+      </c>
+      <c r="I11" s="3" t="inlineStr"/>
       <c r="J11" s="3" t="inlineStr"/>
-      <c r="K11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>3304995000</t>
+          <t>9506996080</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Kosmetické přípravky (lubrikant)</t>
+          <t>Sportovní potřeby (sex stoličky)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>16</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>120</v>
+        <v>67.542</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>90.536</v>
+        <v>75.642</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>101.393</v>
+        <v>1110.74</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>1560.89</v>
-      </c>
-      <c r="I12" s="2" t="n">
-        <v>1767.6</v>
-      </c>
+        <v>1257.84</v>
+      </c>
+      <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr"/>
-      <c r="K12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>9506996080</t>
+          <t>7020006000</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Sportovní potřeby (sex stoličky)</t>
+          <t>Skleněné výrobky (dilda)</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -1015,38 +954,33 @@
           <t>CN</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
+      <c r="D13" s="3" t="n">
+        <v>92</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>16</v>
+        <v>21.232</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>67.542</v>
+        <v>23.778</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>75.642</v>
+        <v>867.9</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>1110.74</v>
-      </c>
-      <c r="I13" s="3" t="n">
-        <v>1257.84</v>
-      </c>
+        <v>982.84</v>
+      </c>
+      <c r="I13" s="3" t="inlineStr"/>
       <c r="J13" s="3" t="inlineStr"/>
-      <c r="K13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>7020006000</t>
+          <t>9403509080</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Skleněné výrobky (dilda)</t>
+          <t>Dřevěný nábytek (bondage stůl)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1054,38 +988,33 @@
           <t>CN</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
+      <c r="D14" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>92</v>
+        <v>53.977</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>21.232</v>
+        <v>60.45</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>23.778</v>
+        <v>752.9299999999999</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>867.9</v>
-      </c>
-      <c r="I14" s="2" t="n">
-        <v>982.84</v>
-      </c>
+        <v>852.64</v>
+      </c>
+      <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr"/>
-      <c r="K14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>9403509080</t>
+          <t>9401616011</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Dřevěný nábytek (bondage stůl)</t>
+          <t>Čalouněná sedadla s dřevěnou kostrou</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -1093,38 +1022,33 @@
           <t>CN</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
+      <c r="D15" s="3" t="n">
+        <v>2</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>4</v>
+        <v>56.3</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>53.977</v>
+        <v>63.051</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>60.45</v>
+        <v>707.52</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>752.9299999999999</v>
-      </c>
-      <c r="I15" s="3" t="n">
-        <v>852.64</v>
-      </c>
+        <v>801.22</v>
+      </c>
+      <c r="I15" s="3" t="inlineStr"/>
       <c r="J15" s="3" t="inlineStr"/>
-      <c r="K15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>9401616011</t>
+          <t>6505009089</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Čalouněná sedadla s dřevěnou kostrou</t>
+          <t>Pokrývky hlavy (masky)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1132,38 +1056,33 @@
           <t>CN</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
+      <c r="D16" s="2" t="n">
+        <v>72</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>2</v>
+        <v>3.216</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>56.3</v>
+        <v>3.602</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>63.051</v>
+        <v>551.45</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>707.52</v>
-      </c>
-      <c r="I16" s="2" t="n">
-        <v>801.22</v>
-      </c>
+        <v>624.48</v>
+      </c>
+      <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr"/>
-      <c r="K16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>6505009089</t>
+          <t>8205700060</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Pokrývky hlavy (masky)</t>
+          <t>Ruční nástroje (klipy na bradavky)</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -1171,124 +1090,109 @@
           <t>CN</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
+      <c r="D17" s="3" t="n">
+        <v>84</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>72</v>
+        <v>5.4</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>3.216</v>
+        <v>6.048</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>3.602</v>
+        <v>533.33</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>551.45</v>
-      </c>
-      <c r="I17" s="3" t="n">
-        <v>624.48</v>
-      </c>
+        <v>603.96</v>
+      </c>
+      <c r="I17" s="3" t="inlineStr"/>
       <c r="J17" s="3" t="inlineStr"/>
-      <c r="K17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>8205700060</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Ruční nástroje (klipy na bradavky)</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="n">
-        <v>84</v>
-      </c>
-      <c r="F18" s="2" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="G18" s="2" t="n">
-        <v>6.048</v>
-      </c>
-      <c r="H18" s="2" t="n">
-        <v>533.33</v>
-      </c>
-      <c r="I18" s="2" t="n">
-        <v>603.96</v>
-      </c>
-      <c r="J18" s="2" t="inlineStr"/>
-      <c r="K18" s="2" t="inlineStr"/>
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>3406000000</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Svíčky</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>120</v>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>15.54</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>17.404</v>
+      </c>
+      <c r="G18" s="5" t="n">
+        <v>505.04</v>
+      </c>
+      <c r="H18" s="5" t="n">
+        <v>571.92</v>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>ANTIDUMPING</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>Antidumpingové clo z CN! Základ A00: 11 990 CZK @ 60,3% = 7 230 CZK + základ 19 220 CZK @ 21% = 2 518 CZK. Ověřit výši při podání JSD.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>3406000000</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>Svíčky</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="n">
-        <v>120</v>
-      </c>
-      <c r="F19" s="5" t="n">
-        <v>15.54</v>
-      </c>
-      <c r="G19" s="5" t="n">
-        <v>17.404</v>
-      </c>
-      <c r="H19" s="5" t="n">
-        <v>505.04</v>
-      </c>
-      <c r="I19" s="5" t="n">
-        <v>571.92</v>
-      </c>
-      <c r="J19" s="5" t="inlineStr">
-        <is>
-          <t>ANTIDUMPING</t>
-        </is>
-      </c>
-      <c r="K19" s="5" t="inlineStr">
-        <is>
-          <t>Antidumpingové clo z CN! Základ A00: 11 990 CZK @ 60,3% = 7 230 CZK + základ 19 220 CZK @ 21% = 2 518 CZK. Ověřit výši při podání JSD.</t>
-        </is>
-      </c>
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>6602000000</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Biče a švihadla</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>7.656</v>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>8.574</v>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>462.44</v>
+      </c>
+      <c r="H19" s="3" t="n">
+        <v>523.6799999999999</v>
+      </c>
+      <c r="I19" s="3" t="inlineStr"/>
+      <c r="J19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>6602000000</t>
+          <t>9020006000</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Biče a švihadla</t>
+          <t>Dýchací přístroje (masky)</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1296,202 +1200,177 @@
           <t>CN</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
+      <c r="D20" s="2" t="n">
+        <v>18</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>24</v>
+        <v>12.924</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>7.656</v>
+        <v>14.474</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>8.574</v>
+        <v>424.24</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>462.44</v>
-      </c>
-      <c r="I20" s="2" t="n">
-        <v>523.6799999999999</v>
-      </c>
+        <v>480.42</v>
+      </c>
+      <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr"/>
-      <c r="K20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>9020006000</t>
+          <t>7325100080</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Dýchací přístroje (masky)</t>
+          <t>Odlitky z oceli (spekulum)</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>15</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>18</v>
+        <v>6.66</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>12.924</v>
+        <v>7.459</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>14.474</v>
+        <v>406.51</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>424.24</v>
-      </c>
-      <c r="I21" s="3" t="n">
-        <v>480.42</v>
-      </c>
+        <v>460.35</v>
+      </c>
+      <c r="I21" s="3" t="inlineStr"/>
       <c r="J21" s="3" t="inlineStr"/>
-      <c r="K21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>7325100080</t>
+          <t>9404902090</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Odlitky z oceli (spekulum)</t>
+          <t>Lůžkoviny (polštáře)</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>9</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>15</v>
+        <v>8.1</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>6.66</v>
+        <v>9.071</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>7.459</v>
+        <v>382.35</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>406.51</v>
-      </c>
-      <c r="I22" s="2" t="n">
-        <v>460.35</v>
-      </c>
+        <v>432.99</v>
+      </c>
+      <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="inlineStr"/>
-      <c r="K22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>9404902090</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>Lůžkoviny (polštáře)</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="F23" s="3" t="n">
-        <v>8.1</v>
-      </c>
-      <c r="G23" s="3" t="n">
-        <v>9.071</v>
-      </c>
-      <c r="H23" s="3" t="n">
-        <v>382.35</v>
-      </c>
-      <c r="I23" s="3" t="n">
-        <v>432.99</v>
-      </c>
-      <c r="J23" s="3" t="inlineStr"/>
-      <c r="K23" s="3" t="inlineStr"/>
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>7616995190</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Výrobky z hliníku (kolíky)</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>4.704</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>5.268</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>297.2</v>
+      </c>
+      <c r="H23" s="4" t="n">
+        <v>336.56</v>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>CBAM</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>CBAM zboží (hliník). Zákazník uplatňuje výjimku de minimis (kód Y137) – dovoz v řádu desítek kg, pod limitem 50 t/rok.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>7616995190</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>Výrobky z hliníku (kolíky)</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="n">
-        <v>56</v>
-      </c>
-      <c r="F24" s="4" t="n">
-        <v>4.704</v>
-      </c>
-      <c r="G24" s="4" t="n">
-        <v>5.268</v>
-      </c>
-      <c r="H24" s="4" t="n">
-        <v>297.2</v>
-      </c>
-      <c r="I24" s="4" t="n">
-        <v>336.56</v>
-      </c>
-      <c r="J24" s="4" t="inlineStr">
-        <is>
-          <t>CBAM</t>
-        </is>
-      </c>
-      <c r="K24" s="4" t="inlineStr">
-        <is>
-          <t>CBAM zboží (hliník). Zákazník uplatňuje výjimku de minimis (kód Y137) – dovoz v řádu desítek kg, pod limitem 50 t/rok.</t>
-        </is>
-      </c>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>8543709860</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Elektrické přístroje (e-stim)</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>3.36</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>203.99</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>231</v>
+      </c>
+      <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>8543709860</t>
+          <t>9503000090</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Elektrické přístroje (e-stim)</t>
+          <t>Hračky (plyšáci, pouta)</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -1499,38 +1378,33 @@
           <t>CN</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
+      <c r="D25" s="3" t="n">
+        <v>30</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>12</v>
+        <v>4.608</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>3</v>
+        <v>5.161</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>3.36</v>
+        <v>199.59</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>203.99</v>
-      </c>
-      <c r="I25" s="3" t="n">
-        <v>231</v>
-      </c>
+        <v>226.02</v>
+      </c>
+      <c r="I25" s="3" t="inlineStr"/>
       <c r="J25" s="3" t="inlineStr"/>
-      <c r="K25" s="3" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>9503000090</t>
+          <t>9401790050</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Hračky (plyšáci, pouta)</t>
+          <t>Ostatní sedadla</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1538,38 +1412,33 @@
           <t>CN</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
+      <c r="D26" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>30</v>
+        <v>6.237</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>4.608</v>
+        <v>6.985</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>5.161</v>
+        <v>176.87</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>199.59</v>
-      </c>
-      <c r="I26" s="2" t="n">
-        <v>226.02</v>
-      </c>
+        <v>200.29</v>
+      </c>
+      <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr"/>
-      <c r="K26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>9401790050</t>
+          <t>8505110090</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Ostatní sedadla</t>
+          <t>Magnety (magnetické kuličky)</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -1577,38 +1446,33 @@
           <t>CN</t>
         </is>
       </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
+      <c r="D27" s="3" t="n">
+        <v>30</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>1</v>
+        <v>0.84</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>6.237</v>
+        <v>0.9409999999999999</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>6.985</v>
+        <v>172.46</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>176.87</v>
-      </c>
-      <c r="I27" s="3" t="n">
-        <v>200.29</v>
-      </c>
+        <v>195.3</v>
+      </c>
+      <c r="I27" s="3" t="inlineStr"/>
       <c r="J27" s="3" t="inlineStr"/>
-      <c r="K27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>8505110090</t>
+          <t>3401115000</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Magnety (magnetické kuličky)</t>
+          <t>Mýdlo</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -1616,169 +1480,111 @@
           <t>CN</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
+      <c r="D28" s="2" t="n">
+        <v>12</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>30</v>
+        <v>3.864</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0.84</v>
+        <v>4.327</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>0.9409999999999999</v>
+        <v>56.37</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>172.46</v>
-      </c>
-      <c r="I28" s="2" t="n">
-        <v>195.3</v>
-      </c>
+        <v>63.84</v>
+      </c>
+      <c r="I28" s="2" t="inlineStr"/>
       <c r="J28" s="2" t="inlineStr"/>
-      <c r="K28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>3401115000</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>Mýdlo</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>FOB (nepotvrzeno)</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="F29" s="3" t="n">
-        <v>3.864</v>
-      </c>
-      <c r="G29" s="3" t="n">
-        <v>4.327</v>
-      </c>
-      <c r="H29" s="3" t="n">
-        <v>56.37</v>
-      </c>
-      <c r="I29" s="3" t="n">
-        <v>63.84</v>
-      </c>
-      <c r="J29" s="3" t="inlineStr"/>
-      <c r="K29" s="3" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="6" t="inlineStr">
+      <c r="A29" s="6" t="inlineStr">
         <is>
           <t>CELKEM</t>
         </is>
       </c>
-      <c r="B30" s="6" t="n"/>
-      <c r="C30" s="6" t="n"/>
-      <c r="D30" s="6" t="n"/>
-      <c r="E30" s="6" t="n">
+      <c r="B29" s="6" t="n"/>
+      <c r="C29" s="6" t="n"/>
+      <c r="D29" s="6" t="n">
         <v>5703</v>
       </c>
-      <c r="F30" s="6" t="n">
+      <c r="E29" s="6" t="n">
         <v>3455.646</v>
       </c>
-      <c r="G30" s="6" t="n">
+      <c r="F29" s="6" t="n">
         <v>3870.045</v>
       </c>
-      <c r="H30" s="6" t="n">
+      <c r="G29" s="6" t="n">
         <v>100229.39</v>
       </c>
-      <c r="I30" s="6" t="n">
+      <c r="H29" s="6" t="n">
         <v>113503.04</v>
       </c>
-      <c r="J30" s="6" t="n"/>
-      <c r="K30" s="6" t="n"/>
+      <c r="I29" s="6" t="n"/>
+      <c r="J29" s="6" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>Legenda:</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="7" t="inlineStr">
-        <is>
-          <t>Legenda:</t>
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>🟡 ORANŽOVÁ</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>CBAM zboží – nutno uvést kód Y137 (de minimis výjimka) v JSD</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>🟡 ORANŽOVÁ</t>
+          <t>🔴 ČERVENÁ</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>CBAM zboží – nutno uvést kód Y137 (de minimis výjimka) v JSD</t>
+          <t>Antidumpingové clo – nutno zkontrolovat a uvést v JSD</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
-          <t>🔴 ČERVENÁ</t>
+          <t>Hrubá hmotnost</t>
         </is>
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>Antidumpingové clo – nutno zkontrolovat a uvést v JSD</t>
+          <t>Vypočtena proporcionálně: čistá hmotnost × 1.11992 (celková GW 3870.05 / celková NW 3455.65)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>FOB (nepotvrzeno)</t>
+          <t>Sleva</t>
         </is>
       </c>
       <c r="B35" s="9" t="inlineStr">
         <is>
-          <t>Incoterm nebyl výslovně uveden v dokumentech – potvrdit s dodavatelem</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr">
-        <is>
-          <t>Hrubá hmotnost</t>
-        </is>
-      </c>
-      <c r="B36" s="9" t="inlineStr">
-        <is>
-          <t>Vypočtena proporcionálně: čistá hmotnost × 1.11992 (celková GW 3870.05 / celková NW 3455.65)</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="8" t="inlineStr">
-        <is>
-          <t>Sleva</t>
-        </is>
-      </c>
-      <c r="B37" s="9" t="inlineStr">
-        <is>
           <t>Obchodní sleva –$13 273,65 z faktury str. 7, faktor 0.883055</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="B35:K35"/>
-    <mergeCell ref="B34:K34"/>
-    <mergeCell ref="B33:K33"/>
-    <mergeCell ref="B36:K36"/>
-    <mergeCell ref="B37:K37"/>
+  <mergeCells count="4">
+    <mergeCell ref="B34:J34"/>
+    <mergeCell ref="B33:J33"/>
+    <mergeCell ref="B35:J35"/>
+    <mergeCell ref="B32:J32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>